<commit_message>
Fixed AML Indicator KL
</commit_message>
<xml_diff>
--- a/reference docs/AML-indicator-KL.xlsx
+++ b/reference docs/AML-indicator-KL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benjz\repos\IMI-Big-Data-AI-AML-Detection-System\reference docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{461F5470-3E13-4B81-8F89-8F696AFDC639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4DB2DC1-3232-4A04-9682-185A89CB6D90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="4" r:id="rId1"/>
@@ -304,9 +304,6 @@
     <t>Card</t>
   </si>
   <si>
-    <t>PROD-008, ACCT-004, PROF-001</t>
-  </si>
-  <si>
     <t>May indicate identity theft</t>
   </si>
   <si>
@@ -325,9 +322,6 @@
     <t>Key investigation trigger</t>
   </si>
   <si>
-    <t>PROD-008</t>
-  </si>
-  <si>
     <t>Products &amp; Services</t>
   </si>
   <si>
@@ -395,9 +389,6 @@
   </si>
   <si>
     <t>Client appears to be living beyond their means; significantly more spending than income</t>
-  </si>
-  <si>
-    <t>PROF-002, PROD-008, HT-SEX-03</t>
   </si>
   <si>
     <t>May indicate proceeds of crime</t>
@@ -1121,6 +1112,15 @@
   </si>
   <si>
     <t>- 5 new general (mostly non-OCG specific) AML typologies have been identified, and the indicators classified under these 5 typologies</t>
+  </si>
+  <si>
+    <t>PROD-001</t>
+  </si>
+  <si>
+    <t>PROF-002, PROD-001, HT-SEX-03</t>
+  </si>
+  <si>
+    <t>PROD-001, ACCT-004, PROF-001</t>
   </si>
 </sst>
 </file>
@@ -1608,6 +1608,45 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1625,45 +1664,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="19" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="19" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="18" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1973,142 +1973,142 @@
   <dimension ref="B2:G16"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2" style="28" customWidth="1"/>
-    <col min="2" max="2" width="22" style="28" customWidth="1"/>
-    <col min="3" max="3" width="52" style="28" customWidth="1"/>
-    <col min="4" max="6" width="18" style="28" customWidth="1"/>
-    <col min="7" max="7" width="22.453125" style="28" customWidth="1"/>
-    <col min="8" max="16384" width="8.54296875" style="28"/>
+    <col min="1" max="1" width="2" style="21" customWidth="1"/>
+    <col min="2" max="2" width="22" style="21" customWidth="1"/>
+    <col min="3" max="3" width="52" style="21" customWidth="1"/>
+    <col min="4" max="6" width="18" style="21" customWidth="1"/>
+    <col min="7" max="7" width="22.453125" style="21" customWidth="1"/>
+    <col min="8" max="16384" width="8.54296875" style="21"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="42" t="s">
-        <v>328</v>
-      </c>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
+      <c r="B2" s="34" t="s">
+        <v>325</v>
+      </c>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
     </row>
     <row r="3" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="41" t="s">
-        <v>329</v>
-      </c>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="39"/>
-      <c r="G3" s="39"/>
+      <c r="B3" s="32" t="s">
+        <v>326</v>
+      </c>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
     </row>
     <row r="4" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="40" t="s">
-        <v>330</v>
-      </c>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
+      <c r="B4" s="37" t="s">
+        <v>327</v>
+      </c>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
     </row>
     <row r="5" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="38">
+      <c r="B6" s="26">
         <v>5</v>
       </c>
-      <c r="C6" s="38">
+      <c r="C6" s="26">
         <v>44</v>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="26">
         <v>24</v>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="26">
         <v>17</v>
       </c>
-      <c r="F6" s="38">
+      <c r="F6" s="26">
         <v>3</v>
       </c>
-      <c r="G6" s="38">
+      <c r="G6" s="26">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="37" t="s">
-        <v>331</v>
-      </c>
-      <c r="C7" s="37" t="s">
-        <v>322</v>
-      </c>
-      <c r="D7" s="37" t="s">
-        <v>323</v>
-      </c>
-      <c r="E7" s="37" t="s">
-        <v>324</v>
-      </c>
-      <c r="F7" s="37" t="s">
-        <v>332</v>
-      </c>
-      <c r="G7" s="37" t="s">
-        <v>333</v>
+      <c r="B7" s="25" t="s">
+        <v>328</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>319</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>320</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>321</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>329</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E8" s="43" t="s">
-        <v>338</v>
+      <c r="E8" s="27" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="7" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="10" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="36" t="s">
-        <v>325</v>
-      </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
+      <c r="B10" s="35" t="s">
+        <v>322</v>
+      </c>
+      <c r="C10" s="36"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
     </row>
     <row r="11" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="23" t="s">
+        <v>331</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>332</v>
+      </c>
+      <c r="D11" s="29" t="s">
+        <v>333</v>
+      </c>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B12" s="23" t="s">
+        <v>323</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>324</v>
+      </c>
+      <c r="D12" s="31" t="s">
         <v>334</v>
       </c>
-      <c r="C11" s="31" t="s">
-        <v>335</v>
-      </c>
-      <c r="D11" s="30" t="s">
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+    </row>
+    <row r="14" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="28" t="s">
         <v>336</v>
       </c>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29"/>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B12" s="32" t="s">
-        <v>326</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>327</v>
-      </c>
-      <c r="D12" s="33" t="s">
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B15" s="28" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B16" s="28" t="s">
         <v>337</v>
-      </c>
-      <c r="E12" s="29"/>
-      <c r="F12" s="29"/>
-      <c r="G12" s="29"/>
-    </row>
-    <row r="14" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="44" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B15" s="44" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B16" s="44" t="s">
-        <v>340</v>
       </c>
     </row>
   </sheetData>
@@ -2187,21 +2187,21 @@
       </c>
     </row>
     <row r="2" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="23"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="40"/>
     </row>
     <row r="3" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
@@ -2532,21 +2532,21 @@
       </c>
     </row>
     <row r="11" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="44" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="22"/>
-      <c r="L11" s="22"/>
-      <c r="M11" s="23"/>
+      <c r="B11" s="39"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="39"/>
+      <c r="I11" s="39"/>
+      <c r="J11" s="39"/>
+      <c r="K11" s="39"/>
+      <c r="L11" s="39"/>
+      <c r="M11" s="40"/>
     </row>
     <row r="12" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
@@ -2656,7 +2656,7 @@
         <v>87</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>88</v>
+        <v>341</v>
       </c>
       <c r="J14" s="7" t="s">
         <v>23</v>
@@ -2668,21 +2668,21 @@
         <v>25</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>72</v>
       </c>
       <c r="C15" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>91</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>92</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>18</v>
@@ -2697,7 +2697,7 @@
         <v>21</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J15" s="7" t="s">
         <v>23</v>
@@ -2709,21 +2709,21 @@
         <v>25</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>96</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>98</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>30</v>
@@ -2738,7 +2738,7 @@
         <v>87</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="J16" s="7" t="s">
         <v>23</v>
@@ -2750,21 +2750,21 @@
         <v>25</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>30</v>
@@ -2779,7 +2779,7 @@
         <v>21</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J17" s="7" t="s">
         <v>23</v>
@@ -2791,21 +2791,21 @@
         <v>25</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>30</v>
@@ -2820,7 +2820,7 @@
         <v>21</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J18" s="7" t="s">
         <v>23</v>
@@ -2837,16 +2837,16 @@
     </row>
     <row r="19" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>18</v>
@@ -2855,13 +2855,13 @@
         <v>75</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H19" s="7" t="s">
         <v>21</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J19" s="7" t="s">
         <v>23</v>
@@ -2873,21 +2873,21 @@
         <v>25</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>18</v>
@@ -2902,7 +2902,7 @@
         <v>21</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>119</v>
+        <v>340</v>
       </c>
       <c r="J20" s="7" t="s">
         <v>23</v>
@@ -2914,21 +2914,21 @@
         <v>25</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>18</v>
@@ -2943,7 +2943,7 @@
         <v>21</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="J21" s="7" t="s">
         <v>23</v>
@@ -2955,21 +2955,21 @@
         <v>25</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>46</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>30</v>
@@ -2984,7 +2984,7 @@
         <v>21</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="J22" s="7" t="s">
         <v>23</v>
@@ -2996,44 +2996,44 @@
         <v>25</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="23"/>
+      <c r="A23" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" s="39"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="39"/>
+      <c r="K23" s="39"/>
+      <c r="L23" s="39"/>
+      <c r="M23" s="40"/>
     </row>
     <row r="24" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>132</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>135</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>20</v>
@@ -3042,7 +3042,7 @@
         <v>21</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="J24" s="9" t="s">
         <v>23</v>
@@ -3054,191 +3054,191 @@
         <v>25</v>
       </c>
       <c r="M24" s="9" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>139</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>142</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="H25" s="9" t="s">
         <v>21</v>
       </c>
       <c r="I25" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="K25" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="L25" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="J25" s="9" t="s">
+      <c r="M25" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="K25" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="L25" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="M25" s="9" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="9" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="L26" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="M26" s="9" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="L27" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="M27" s="9" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="9" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>20</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="J28" s="9" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="L28" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="M28" s="9" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="9" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B29" s="9" t="s">
         <v>46</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>20</v>
@@ -3247,7 +3247,7 @@
         <v>21</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="J29" s="9" t="s">
         <v>23</v>
@@ -3259,53 +3259,53 @@
         <v>25</v>
       </c>
       <c r="M29" s="9" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="24" t="s">
-        <v>170</v>
-      </c>
-      <c r="B30" s="22"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
-      <c r="I30" s="22"/>
-      <c r="J30" s="22"/>
-      <c r="K30" s="22"/>
-      <c r="L30" s="22"/>
-      <c r="M30" s="23"/>
+      <c r="A30" s="41" t="s">
+        <v>167</v>
+      </c>
+      <c r="B30" s="39"/>
+      <c r="C30" s="39"/>
+      <c r="D30" s="39"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="39"/>
+      <c r="H30" s="39"/>
+      <c r="I30" s="39"/>
+      <c r="J30" s="39"/>
+      <c r="K30" s="39"/>
+      <c r="L30" s="39"/>
+      <c r="M30" s="40"/>
     </row>
     <row r="31" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="D31" s="11" t="s">
         <v>171</v>
-      </c>
-      <c r="B31" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="D31" s="11" t="s">
-        <v>174</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F31" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="I31" s="11" t="s">
         <v>175</v>
-      </c>
-      <c r="G31" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="H31" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="I31" s="11" t="s">
-        <v>178</v>
       </c>
       <c r="J31" s="11" t="s">
         <v>23</v>
@@ -3317,36 +3317,36 @@
         <v>25</v>
       </c>
       <c r="M31" s="11" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="11" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="E32" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="J32" s="11" t="s">
         <v>23</v>
@@ -3358,36 +3358,36 @@
         <v>25</v>
       </c>
       <c r="M32" s="11" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="11" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="J33" s="11" t="s">
         <v>23</v>
@@ -3399,36 +3399,36 @@
         <v>25</v>
       </c>
       <c r="M33" s="11" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="34" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="11" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="H34" s="11" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="J34" s="11" t="s">
         <v>23</v>
@@ -3440,36 +3440,36 @@
         <v>25</v>
       </c>
       <c r="M34" s="11" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="35" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="11" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F35" s="12" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H35" s="11" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="J35" s="11" t="s">
         <v>23</v>
@@ -3481,36 +3481,36 @@
         <v>25</v>
       </c>
       <c r="M35" s="11" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="36" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="D36" s="11" t="s">
         <v>205</v>
-      </c>
-      <c r="B36" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="C36" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="D36" s="11" t="s">
-        <v>208</v>
       </c>
       <c r="E36" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G36" s="11" t="s">
         <v>20</v>
       </c>
       <c r="H36" s="11" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="J36" s="11" t="s">
         <v>23</v>
@@ -3522,36 +3522,36 @@
         <v>25</v>
       </c>
       <c r="M36" s="11" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="37" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="11" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G37" s="11" t="s">
         <v>20</v>
       </c>
       <c r="H37" s="11" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="J37" s="11" t="s">
         <v>23</v>
@@ -3563,44 +3563,44 @@
         <v>25</v>
       </c>
       <c r="M37" s="11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="38" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="25" t="s">
-        <v>217</v>
-      </c>
-      <c r="B38" s="22"/>
-      <c r="C38" s="22"/>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="22"/>
-      <c r="I38" s="22"/>
-      <c r="J38" s="22"/>
-      <c r="K38" s="22"/>
-      <c r="L38" s="22"/>
-      <c r="M38" s="23"/>
+      <c r="A38" s="42" t="s">
+        <v>214</v>
+      </c>
+      <c r="B38" s="39"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="39"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
+      <c r="H38" s="39"/>
+      <c r="I38" s="39"/>
+      <c r="J38" s="39"/>
+      <c r="K38" s="39"/>
+      <c r="L38" s="39"/>
+      <c r="M38" s="40"/>
     </row>
     <row r="39" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="D39" s="13" t="s">
         <v>218</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="C39" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D39" s="13" t="s">
-        <v>221</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G39" s="13" t="s">
         <v>20</v>
@@ -3609,39 +3609,39 @@
         <v>87</v>
       </c>
       <c r="I39" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="J39" s="13" t="s">
+        <v>221</v>
+      </c>
+      <c r="K39" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="L39" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="J39" s="13" t="s">
+      <c r="M39" s="13" t="s">
         <v>224</v>
-      </c>
-      <c r="K39" s="13" t="s">
-        <v>225</v>
-      </c>
-      <c r="L39" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="M39" s="13" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="13" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G40" s="13" t="s">
         <v>20</v>
@@ -3650,39 +3650,39 @@
         <v>87</v>
       </c>
       <c r="I40" s="13" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="J40" s="13" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="K40" s="13" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L40" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="M40" s="13" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="41" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="13" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="E41" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G41" s="13" t="s">
         <v>20</v>
@@ -3691,121 +3691,121 @@
         <v>87</v>
       </c>
       <c r="I41" s="13" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="J41" s="13" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="K41" s="13" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L41" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="M41" s="13" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="42" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="13" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>54</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G42" s="13" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="H42" s="13" t="s">
         <v>87</v>
       </c>
       <c r="I42" s="13" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="J42" s="13" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="K42" s="13" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L42" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="M42" s="13" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="43" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="13" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>54</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G43" s="13" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="H43" s="13" t="s">
         <v>87</v>
       </c>
       <c r="I43" s="13" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="J43" s="13" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="K43" s="13" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L43" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="M43" s="13" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="44" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="13" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F44" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G44" s="13" t="s">
         <v>20</v>
@@ -3814,80 +3814,80 @@
         <v>87</v>
       </c>
       <c r="I44" s="13" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J44" s="13" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="K44" s="13" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L44" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="M44" s="13" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="45" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="13" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E45" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G45" s="13" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="H45" s="13" t="s">
         <v>42</v>
       </c>
       <c r="I45" s="13" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="J45" s="13" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="K45" s="13" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L45" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="M45" s="13" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="46" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="13" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G46" s="13" t="s">
         <v>20</v>
@@ -3896,39 +3896,39 @@
         <v>87</v>
       </c>
       <c r="I46" s="13" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J46" s="13" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="K46" s="13" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L46" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="M46" s="13" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="47" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="13" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E47" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G47" s="13" t="s">
         <v>20</v>
@@ -3937,142 +3937,142 @@
         <v>87</v>
       </c>
       <c r="I47" s="13" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="J47" s="13" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="K47" s="13" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L47" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="M47" s="13" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="48" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="13" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E48" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F48" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G48" s="13" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="H48" s="13" t="s">
         <v>87</v>
       </c>
       <c r="I48" s="13" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="J48" s="13" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="K48" s="13" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L48" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="M48" s="13" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="49" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="13" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="E49" s="5" t="s">
         <v>30</v>
       </c>
       <c r="F49" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="G49" s="13" t="s">
+        <v>273</v>
+      </c>
+      <c r="H49" s="13" t="s">
+        <v>274</v>
+      </c>
+      <c r="I49" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="J49" s="13" t="s">
+        <v>221</v>
+      </c>
+      <c r="K49" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="G49" s="13" t="s">
+      <c r="L49" s="13" t="s">
+        <v>223</v>
+      </c>
+      <c r="M49" s="13" t="s">
         <v>276</v>
-      </c>
-      <c r="H49" s="13" t="s">
-        <v>277</v>
-      </c>
-      <c r="I49" s="13" t="s">
-        <v>278</v>
-      </c>
-      <c r="J49" s="13" t="s">
-        <v>224</v>
-      </c>
-      <c r="K49" s="13" t="s">
-        <v>225</v>
-      </c>
-      <c r="L49" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="M49" s="13" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="50" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="13" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F50" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="G50" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="H50" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="I50" s="13" t="s">
+        <v>280</v>
+      </c>
+      <c r="J50" s="13" t="s">
+        <v>221</v>
+      </c>
+      <c r="K50" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="G50" s="13" t="s">
-        <v>240</v>
-      </c>
-      <c r="H50" s="13" t="s">
-        <v>282</v>
-      </c>
-      <c r="I50" s="13" t="s">
-        <v>283</v>
-      </c>
-      <c r="J50" s="13" t="s">
-        <v>224</v>
-      </c>
-      <c r="K50" s="13" t="s">
-        <v>225</v>
-      </c>
       <c r="L50" s="13" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="M50" s="13" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -4100,17 +4100,17 @@
   <sheetData>
     <row r="1" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="15" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
     </row>
     <row r="2" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="16" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C2" s="16"/>
     </row>
@@ -4119,7 +4119,7 @@
         <v>30</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C3" s="18"/>
     </row>
@@ -4128,7 +4128,7 @@
         <v>18</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C4" s="18"/>
     </row>
@@ -4137,7 +4137,7 @@
         <v>54</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C5" s="18"/>
     </row>
@@ -4148,7 +4148,7 @@
     </row>
     <row r="7" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
@@ -4158,10 +4158,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
@@ -4169,10 +4169,10 @@
         <v>19</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
@@ -4180,43 +4180,43 @@
         <v>75</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="18" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="18" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="18" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
@@ -4226,17 +4226,17 @@
     </row>
     <row r="15" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
     </row>
     <row r="16" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>12</v>
@@ -4247,10 +4247,10 @@
         <v>62</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
@@ -4258,65 +4258,65 @@
         <v>87</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="18" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="18" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="18" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="18" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="18" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
   </sheetData>

</xml_diff>